<commit_message>
added new user rank
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -16,7 +16,7 @@
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-08-16 to 2026-08-22</t>
+    <t>2026-09-06 to 2026-09-12</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -583,7 +583,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -594,10 +594,10 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -605,7 +605,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -616,10 +616,10 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -627,7 +627,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -638,7 +638,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -649,10 +649,10 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -660,10 +660,10 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -685,7 +685,7 @@
         <v>4</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -693,10 +693,10 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -726,10 +726,10 @@
         <v>20</v>
       </c>
       <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20">
         <v>1</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -737,7 +737,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -751,7 +751,7 @@
         <v>4</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -759,10 +759,10 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C23">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,10 +792,10 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -803,10 +803,10 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -814,7 +814,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -847,10 +847,10 @@
         <v>31</v>
       </c>
       <c r="B31">
+        <v>4</v>
+      </c>
+      <c r="C31">
         <v>1</v>
-      </c>
-      <c r="C31">
-        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -858,7 +858,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -891,7 +891,7 @@
         <v>35</v>
       </c>
       <c r="B35">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C35">
         <v>0</v>
@@ -902,7 +902,7 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C36">
         <v>0</v>
@@ -913,7 +913,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C37">
         <v>1</v>

</xml_diff>

<commit_message>
addition of pharmaceutical care plan documentation - start of UI and basic backend
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -16,7 +16,7 @@
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-09-06 to 2026-09-12</t>
+    <t>2026-10-11 to 2026-10-17</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -82,9 +82,6 @@
     <t>SAMUEL Onyedika Samuel</t>
   </si>
   <si>
-    <t>ABIONA Damilola Peace</t>
-  </si>
-  <si>
     <t>IKUKOYI Dayo Sunday</t>
   </si>
   <si>
@@ -125,6 +122,9 @@
   </si>
   <si>
     <t>AFOLABI Bukola Adejoke</t>
+  </si>
+  <si>
+    <t>OGUNYEMI Temitope Helen</t>
   </si>
 </sst>
 </file>
@@ -561,10 +561,10 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -583,7 +583,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -594,10 +594,10 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -605,10 +605,10 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -616,10 +616,10 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C10">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -627,7 +627,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -649,10 +649,10 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -660,10 +660,10 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -671,7 +671,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -682,10 +682,10 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C16">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -693,10 +693,10 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -715,7 +715,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -726,10 +726,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -748,7 +748,7 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -759,7 +759,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -781,10 +781,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,10 +792,10 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -803,7 +803,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -814,7 +814,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -847,10 +847,10 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C31">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -858,7 +858,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -869,7 +869,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>34</v>
       </c>
       <c r="B34">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -902,10 +902,10 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C36">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -913,10 +913,10 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C37">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
blocking submission of more than 1 report per day
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -16,7 +16,7 @@
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-10-11 to 2026-10-17</t>
+    <t>2026-10-18 to 2026-10-24</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -564,7 +564,7 @@
         <v>4</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -575,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -583,7 +583,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -594,7 +594,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -605,7 +605,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -627,7 +627,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -641,7 +641,7 @@
         <v>4</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -649,7 +649,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -660,10 +660,10 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -671,7 +671,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -682,7 +682,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -715,7 +715,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -726,10 +726,10 @@
         <v>20</v>
       </c>
       <c r="B20">
+        <v>7</v>
+      </c>
+      <c r="C20">
         <v>1</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -737,7 +737,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -748,10 +748,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -759,7 +759,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -784,7 +784,7 @@
         <v>4</v>
       </c>
       <c r="C25">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -792,7 +792,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -803,7 +803,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -814,7 +814,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -858,7 +858,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -869,7 +869,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>34</v>
       </c>
       <c r="B34">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -891,10 +891,10 @@
         <v>35</v>
       </c>
       <c r="B35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C35">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -902,10 +902,10 @@
         <v>36</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -913,7 +913,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C37">
         <v>0</v>

</xml_diff>

<commit_message>
changed curePeriod from 24hrs to 6hrs
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -16,7 +16,7 @@
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-10-18 to 2026-10-24</t>
+    <t>2026-10-24 to 2026-10-30</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -561,10 +561,10 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -572,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -583,7 +583,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -605,7 +605,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -616,10 +616,10 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -641,7 +641,7 @@
         <v>4</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -660,10 +660,10 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -693,10 +693,10 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -704,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -715,7 +715,7 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19">
         <v>0</v>
@@ -726,10 +726,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C20">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -737,7 +737,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -748,10 +748,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -759,7 +759,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C23">
         <v>0</v>
@@ -781,7 +781,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -792,7 +792,7 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C26">
         <v>0</v>
@@ -803,7 +803,7 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C27">
         <v>0</v>
@@ -814,7 +814,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -836,7 +836,7 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -847,7 +847,7 @@
         <v>31</v>
       </c>
       <c r="B31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -858,7 +858,7 @@
         <v>32</v>
       </c>
       <c r="B32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C32">
         <v>0</v>
@@ -869,7 +869,7 @@
         <v>33</v>
       </c>
       <c r="B33">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C33">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>34</v>
       </c>
       <c r="B34">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C34">
         <v>0</v>
@@ -891,7 +891,7 @@
         <v>35</v>
       </c>
       <c r="B35">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -913,7 +913,7 @@
         <v>37</v>
       </c>
       <c r="B37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C37">
         <v>0</v>

</xml_diff>